<commit_message>
Cost of debt = risk-free + 1% (PM decision) and re-run of Diageo
Amanda chose to replace the historic cost of debt (3.81%, below the
5.22% US 10-year) with risk-free + a 1.0% credit spread, now set in the
brief. The engine applies the rule (apply_brief_rules) and keeps the
historic figure for reference. Valuation, bear case and memo re-run:
fair value 2,141p (was 2,475p), WACC 6.75%, still BUY (+28.0%).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DxwbAxWQ7gXdAJQN7iiAbU
</commit_message>
<xml_diff>
--- a/runs/DGE/2026-10-12/valuation/dcf.xlsx
+++ b/runs/DGE/2026-10-12/valuation/dcf.xlsx
@@ -614,11 +614,11 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.03806</v>
+        <v>0.06220000000000001</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) p.211: FY26 net interest charge 812 / average net borrowings 21,336 (historic cost; see notes.md FLAG)</t>
+          <t>risk-free 5.22% + credit spread 1.00% (PM rule, briefs)</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2959.700706318815</v>
+        <v>2890.0898107331</v>
       </c>
     </row>
     <row r="16">
@@ -1288,7 +1288,7 @@
         <v/>
       </c>
       <c r="C18" s="6" t="n">
-        <v>0.02881142</v>
+        <v>0.04708540000000001</v>
       </c>
     </row>
     <row r="19">
@@ -1302,7 +1302,7 @@
         <v/>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.06209361440900001</v>
+        <v>0.06746525083</v>
       </c>
     </row>
     <row r="20">
@@ -1316,7 +1316,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>15032.82659909468</v>
+        <v>14824.93257153591</v>
       </c>
     </row>
     <row r="21">
@@ -1330,7 +1330,7 @@
         <v/>
       </c>
       <c r="C21" s="4" t="n">
-        <v>95293.35043967597</v>
+        <v>84509.01404726508</v>
       </c>
     </row>
     <row r="22">
@@ -1344,7 +1344,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>71718.59111722476</v>
+        <v>62106.3105197913</v>
       </c>
     </row>
     <row r="23">
@@ -1358,7 +1358,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>86751.41771631944</v>
+        <v>76931.24309132721</v>
       </c>
     </row>
     <row r="24">
@@ -1372,7 +1372,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>72788.71771631944</v>
+        <v>62968.54309132721</v>
       </c>
     </row>
     <row r="25">
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>32.75819879222297</v>
+        <v>28.33867825892314</v>
       </c>
     </row>
     <row r="26">
@@ -1400,7 +1400,7 @@
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>2475.305938659738</v>
+        <v>2141.353956394374</v>
       </c>
     </row>
     <row r="27">
@@ -1414,7 +1414,7 @@
         <v/>
       </c>
       <c r="C27" s="6" t="n">
-        <v>0.4795612305</v>
+        <v>0.2799485693</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Evidence-based beta for Diageo: 0.96 bottom-up (PM decision); re-run
Amanda required the beta to be backed by evidence. The Risk agent tested
seven estimates with standard errors and 95% intervals (risk/beta_evidence.py):
the first run's 0.48 came from the noisiest one (s.e. 0.25) and is rejected.
Precise own-regression estimates are 0.60-0.77; the industry bottom-up beta
(Damodaran global alcoholic beverages, unlevered 0.73, relevered at
Diageo's D/E 0.416) is 0.96, which Amanda chose.

Re-run: WACC 8.46%, fair value 1,448p, SELL (-13.5%). Memo restructured.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DxwbAxWQ7gXdAJQN7iiAbU
</commit_message>
<xml_diff>
--- a/runs/DGE/2026-10-12/valuation/dcf.xlsx
+++ b/runs/DGE/2026-10-12/valuation/dcf.xlsx
@@ -599,11 +599,11 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.475</v>
+        <v>0.9601</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Risk agent: peer median 5y monthly beta (Pernod, Remy, Campari, Brown-Forman vs home indices). DGE's own 5y monthly vs FTSE 100 = 0.37, R2=0.04, n=60, rejected as unreliable</t>
+          <t>Risk agent, bottom-up: Damodaran global alcoholic beverages unlevered beta 0.73 (Jan 2026, cash-corrected) relevered at Diageo D/E 0.416, tax 24.3%. See risk/beta_evidence.json</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2890.0898107331</v>
+        <v>2681.030055590724</v>
       </c>
     </row>
     <row r="16">
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.07595</v>
+        <v>0.100205</v>
       </c>
     </row>
     <row r="18">
@@ -1302,7 +1302,7 @@
         <v/>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.06746525083</v>
+        <v>0.08459049358000001</v>
       </c>
     </row>
     <row r="20">
@@ -1316,7 +1316,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>14824.93257153591</v>
+        <v>14192.13468609485</v>
       </c>
     </row>
     <row r="21">
@@ -1330,7 +1330,7 @@
         <v/>
       </c>
       <c r="C21" s="4" t="n">
-        <v>84509.01404726508</v>
+        <v>62102.6613487822</v>
       </c>
     </row>
     <row r="22">
@@ -1344,7 +1344,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>62106.3105197913</v>
+        <v>42338.28393516572</v>
       </c>
     </row>
     <row r="23">
@@ -1358,7 +1358,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>76931.24309132721</v>
+        <v>56530.41862126057</v>
       </c>
     </row>
     <row r="24">
@@ -1372,7 +1372,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>62968.54309132721</v>
+        <v>42567.71862126057</v>
       </c>
     </row>
     <row r="25">
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>28.33867825892314</v>
+        <v>19.15738911847911</v>
       </c>
     </row>
     <row r="26">
@@ -1400,7 +1400,7 @@
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>2141.353956394374</v>
+        <v>1447.588719848807</v>
       </c>
     </row>
     <row r="27">
@@ -1414,7 +1414,7 @@
         <v/>
       </c>
       <c r="C27" s="6" t="n">
-        <v>0.2799485693</v>
+        <v>-0.1347347759</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phase 3 re-run: Valuation agent (1,524p HOLD)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015cJiGSSnTAwJQDY1YEwHLn
</commit_message>
<xml_diff>
--- a/runs/DGE/2026-10-12/valuation/dcf.xlsx
+++ b/runs/DGE/2026-10-12/valuation/dcf.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -535,268 +535,328 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Net working capital % of sales</t>
+          <t>Terminal-year capex % of sales</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.37576</v>
+        <v>0.06211688111691262</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FY26 (inventories incl. maturing 10,529 + trade &amp; other receivables 3,277 - trade &amp; other payables 6,425) / net sales 19,643; Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) balance sheet</t>
+          <t>PM rule: return on new investment 13.4% (value driver formula, briefs/DGE.yaml)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Savings flow-through</t>
+          <t>Net working capital % of sales</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.5</v>
+        <v>0.37576</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PM assumption (briefs/DGE.yaml)</t>
+          <t>FY26 (inventories incl. maturing 10,529 + trade &amp; other receivables 3,277 - trade &amp; other payables 6,425) / net sales 19,643; Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) balance sheet</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Risk-free rate (US 10y)</t>
+          <t>Savings flow-through</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.0522</v>
+        <v>0.46</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FRED DGS10 (US 10-year Treasury, constant maturity), 2026-10-08</t>
+          <t>PM assumption (briefs/DGE.yaml)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Equity risk premium</t>
+          <t>Risk-free rate (US 10y)</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.05</v>
+        <v>0.0522</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PM assumption (briefs/DGE.yaml)</t>
+          <t>FRED DGS10 (US 10-year Treasury, constant maturity), 2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Beta</t>
+          <t>Equity risk premium</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.9601</v>
+        <v>0.05</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Risk agent, bottom-up: Damodaran global alcoholic beverages unlevered beta 0.73 (Jan 2026, cash-corrected) relevered at Diageo D/E 0.416, tax 24.3%. See risk/beta_evidence.json</t>
+          <t>PM assumption (briefs/DGE.yaml)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Pre-tax cost of debt</t>
+          <t>Beta</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.06220000000000001</v>
+        <v>0.9601</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>risk-free 5.22% + credit spread 1.00% (PM rule, briefs)</t>
+          <t>Risk agent, bottom-up: Damodaran global alcoholic beverages unlevered beta 0.73 (Jan 2026, cash-corrected) relevered at Diageo D/E 0.416, tax 24.3%. See risk/beta_evidence.json</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Debt weight D/(D+E)</t>
+          <t>Pre-tax cost of debt</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0.29395</v>
+        <v>0.06220000000000001</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>net debt 20,482 / (net debt + market cap 49,196 = 2,222m shares x 1673p x 1.3234 USD/GBP)</t>
+          <t>risk-free 5.22% + credit spread 1.00% (PM rule, briefs)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Terminal growth</t>
+          <t>Debt weight D/(D+E)</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.02</v>
+        <v>0.29395</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PM assumption (briefs/DGE.yaml)</t>
+          <t>net debt 20,482 / (net debt + market cap 49,196 = 2,222m shares x 1673p x 1.3234 USD/GBP)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Fraction of FY27 elapsed at valuation date</t>
+          <t>Terminal growth</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.2822</v>
+        <v>0.02</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>103 days of FY27 (from 1 Jul 2026) elapsed at run date 2026-10-12 / 365</t>
+          <t>PM assumption (briefs/DGE.yaml)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Net debt (USD m)</t>
+          <t>Fraction of FY27 elapsed, used in discounting (0 = valued at 30 June)</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>20482</v>
+        <v>0</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 17 p.187: net borrowings 20,482 (INCLUDES lease liabilities 685; EABL/RCB loans of 272 sit in liabilities held for sale)</t>
+          <t>103 days of FY27 (from 1 Jul 2026) elapsed at run date 2026-10-12 / 365</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lease liabilities not in net debt (USD m)</t>
+          <t>Years from 30 June to valuation date (equity roll-forward)</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>0</v>
+        <v>0.2822</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0 because the 685 of lease liabilities is already inside net borrowings (20-F note 17 p.187)</t>
+          <t>103 days of FY27 (from 1 Jul 2026) elapsed at run date 2026-10-12 / 365</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Minority interests (USD m)</t>
+          <t>Dividends gone ex before valuation date (USD m)</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>2083</v>
+        <v>0</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) balance sheet, non-controlling interests at book value (USL 755, other 1,328: p.189)</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529): FY26 final dividend 30c, ex-dividend 15 October 2026 (ordinary shares), AFTER the 12 Oct 2026 valuation date, so the 1,673p price is cum-dividend and nothing is deducted. No other dividend went ex between 30 June and 12 Oct 2026.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Pension deficit (USD m)</t>
+          <t>Net debt (USD m)</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>0</v>
+        <v>20482</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18): net post-employment SURPLUS 627 (XBRL LiabilityAssetOfDefinedBenefitPlans -627); brief rule: 0 if in surplus. Deficit plans alone: 387 (see FLAG)</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 17 p.187: net borrowings 20,482 (INCLUDES lease liabilities 685; EABL/RCB loans of 272 sit in liabilities held for sale)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Associates incl. Moet Hennessy (USD m)</t>
+          <t>Lease liabilities not in net debt (USD m)</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>5284</v>
+        <v>0</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 'Investments in associates': Moet Hennessy 34% at 5,107 (carrying value tested at fair value less costs of disposal, 'sensitive' = little headroom) + others 177</t>
+          <t>0 because the 685 of lease liabilities is already inside net borrowings (20-F note 17 p.187)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Disposal proceeds not in net debt (USD m)</t>
+          <t>Minority interests (USD m)</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>3318.3</v>
+        <v>2083</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>EABL + Kenyan spirits sale to Asahi c.$2.3bn (20-F p.85) + Diageo's 57.21% of USL's RCB sale INR 166.6bn = c.$1.78bn (USL/press, 24 Mar 2026); both gross, before tax and costs, not in net debt at 30 June 2026</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) balance sheet, non-controlling interests at book value (USL 755, other 1,328: p.189)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ordinary shares (m)</t>
+          <t>Pension deficit (USD m)</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>2222</v>
+        <v>0</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) p.188 and XBRL: 2,432m issued - 208m treasury - 2m employee trusts (ordinary shares, NOT ADRs)</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18): net post-employment SURPLUS 627 (XBRL LiabilityAssetOfDefinedBenefitPlans -627); brief rule: 0 if in surplus. Deficit plans alone: 387 (see FLAG)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>USD per GBP</t>
+          <t>Associates incl. Moet Hennessy (USD m)</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>1.3234</v>
+        <v>5284</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FRED DEXUSUK (USD per GBP, noon buying rate New York), 2026-10-02</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 'Investments in associates': Moet Hennessy 34% at 5,107 (carrying value tested at fair value less costs of disposal, 'sensitive' = little headroom) + others 177</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Disposal proceeds not in net debt (USD m)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>3318.3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>EABL + Kenyan spirits sale to Asahi c.$2.3bn (20-F p.85) + Diageo's 57.21% of USL's RCB sale INR 166.6bn = c.$1.78bn (USL/press, 24 Mar 2026); both gross, before tax and costs, not in net debt at 30 June 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Restructuring cash still to pay (USD m)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>850</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Diageo Capital Markets Day 6-K, 6 Aug 2026 (SEC accession 0001654954-26-007324): c.$800m exceptional cash costs for the operating framework + c.$50m for supply chain in FY27; FY27-29 cumulative free cash flow c.$8bn after c.$850m exceptional cash costs (also 20-F FY26 CEO letter). Pre-tax, undiscounted: any tax relief (up to c.$207m at 24.3%) is not confirmed, so not counted. Not in net debt at 30 June 2026; the forecast is before exceptionals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Ordinary shares (m)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>2222</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) p.188 and XBRL: 2,432m issued - 208m treasury - 2m employee trusts (ordinary shares, NOT ADRs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>USD per GBP</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1.3234</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>FRED DEXUSUK (USD per GBP, noon buying rate New York), 2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Share price (pence)</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B28" s="2" t="n">
         <v>1673</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Yahoo Finance DGE.L close (pence, GBp), 2026-10-12</t>
         </is>
@@ -813,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -925,23 +985,23 @@
         </is>
       </c>
       <c r="C4" s="4">
-        <f>377.5*Inputs!$B$8</f>
+        <f>377.5*Inputs!$B$9</f>
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>962.5*Inputs!$B$8</f>
+        <f>962.5*Inputs!$B$9</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>1000.0*Inputs!$B$8</f>
+        <f>1000.0*Inputs!$B$9</f>
         <v/>
       </c>
       <c r="F4" s="4">
-        <f>1000.0*Inputs!$B$8</f>
+        <f>1000.0*Inputs!$B$9</f>
         <v/>
       </c>
       <c r="G4" s="4">
-        <f>1000.0*Inputs!$B$8</f>
+        <f>1000.0*Inputs!$B$9</f>
         <v/>
       </c>
     </row>
@@ -972,7 +1032,7 @@
         <v/>
       </c>
       <c r="I5" s="4" t="n">
-        <v>6496.414518235197</v>
+        <v>6456.414518235197</v>
       </c>
     </row>
     <row r="6">
@@ -1090,23 +1150,23 @@
         </is>
       </c>
       <c r="C10" s="4">
-        <f>(C3-B3)*Inputs!$B$7</f>
+        <f>(C3-B3)*Inputs!$B$8</f>
         <v/>
       </c>
       <c r="D10" s="4">
-        <f>(D3-C3)*Inputs!$B$7</f>
+        <f>(D3-C3)*Inputs!$B$8</f>
         <v/>
       </c>
       <c r="E10" s="4">
-        <f>(E3-D3)*Inputs!$B$7</f>
+        <f>(E3-D3)*Inputs!$B$8</f>
         <v/>
       </c>
       <c r="F10" s="4">
-        <f>(F3-E3)*Inputs!$B$7</f>
+        <f>(F3-E3)*Inputs!$B$8</f>
         <v/>
       </c>
       <c r="G10" s="4">
-        <f>(G3-F3)*Inputs!$B$7</f>
+        <f>(G3-F3)*Inputs!$B$8</f>
         <v/>
       </c>
     </row>
@@ -1137,7 +1197,7 @@
         <v/>
       </c>
       <c r="I11" s="4" t="n">
-        <v>3932.589754068069</v>
+        <v>3902.30975406807</v>
       </c>
     </row>
     <row r="12">
@@ -1147,7 +1207,7 @@
         </is>
       </c>
       <c r="C12" s="4">
-        <f>C11*(1-Inputs!$B$15)</f>
+        <f>C11*(1-Inputs!$B$16)</f>
         <v/>
       </c>
       <c r="D12" s="4">
@@ -1174,23 +1234,23 @@
         </is>
       </c>
       <c r="C13" s="5">
-        <f>1-Inputs!$B$15</f>
+        <f>1-Inputs!$B$16</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>2-Inputs!$B$15</f>
+        <f>2-Inputs!$B$16</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>3-Inputs!$B$15</f>
+        <f>3-Inputs!$B$16</f>
         <v/>
       </c>
       <c r="F13" s="5">
-        <f>4-Inputs!$B$15</f>
+        <f>4-Inputs!$B$16</f>
         <v/>
       </c>
       <c r="G13" s="5">
-        <f>5-Inputs!$B$15</f>
+        <f>5-Inputs!$B$16</f>
         <v/>
       </c>
     </row>
@@ -1248,7 +1308,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2681.030055590724</v>
+        <v>2600.116287717255</v>
       </c>
     </row>
     <row r="16">
@@ -1270,7 +1330,7 @@
         </is>
       </c>
       <c r="B17" s="6">
-        <f>Inputs!$B$9+Inputs!$B$11*Inputs!$B$10</f>
+        <f>Inputs!$B$10+Inputs!$B$12*Inputs!$B$11</f>
         <v/>
       </c>
       <c r="C17" s="6" t="n">
@@ -1284,7 +1344,7 @@
         </is>
       </c>
       <c r="B18" s="6">
-        <f>Inputs!$B$12*(1-Inputs!$B$4)</f>
+        <f>Inputs!$B$13*(1-Inputs!$B$4)</f>
         <v/>
       </c>
       <c r="C18" s="6" t="n">
@@ -1298,7 +1358,7 @@
         </is>
       </c>
       <c r="B19" s="6">
-        <f>(1-Inputs!$B$13)*B17+Inputs!$B$13*B18</f>
+        <f>(1-Inputs!$B$14)*B17+Inputs!$B$14*B18</f>
         <v/>
       </c>
       <c r="C19" s="6" t="n">
@@ -1316,105 +1376,133 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>14192.13468609485</v>
+        <v>14697.21172715634</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Terminal value (Gordon growth)</t>
+          <t>Terminal-year FCF (normalised, grows at g)</t>
         </is>
       </c>
       <c r="B21" s="4">
-        <f>G11*(1+Inputs!$B$14)/(WACC-Inputs!$B$14)</f>
+        <f>G7*(1+Inputs!$B$15)+G3*(1+Inputs!$B$15)*Inputs!$B$5-G3*(1+Inputs!$B$15)*Inputs!$B$7-G3*Inputs!$B$15*Inputs!$B$8</f>
         <v/>
       </c>
       <c r="C21" s="4" t="n">
-        <v>62102.6613487822</v>
+        <v>4241.187860422046</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PV of terminal value</t>
+          <t>Terminal value (Gordon growth)</t>
         </is>
       </c>
       <c r="B22" s="4">
-        <f>B21/(1+WACC)^(5-Inputs!$B$15)</f>
+        <f>B21/(WACC-Inputs!$B$15)</f>
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>42338.28393516572</v>
+        <v>65662.7256636308</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Enterprise value</t>
+          <t>PV of terminal value</t>
         </is>
       </c>
       <c r="B23" s="4">
-        <f>B20+B22</f>
+        <f>B22/(1+WACC)^(5-Inputs!$B$16)</f>
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>56530.41862126057</v>
+        <v>43751.19692021715</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Equity value</t>
+          <t>Enterprise value</t>
         </is>
       </c>
       <c r="B24" s="4">
-        <f>B23-Inputs!$B$16-Inputs!$B$17-Inputs!$B$18-Inputs!$B$19+Inputs!$B$20+Inputs!$B$21</f>
+        <f>B20+B23</f>
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>42567.71862126057</v>
+        <v>58448.40864737349</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Value per share (USD)</t>
+          <t>Equity value at balance sheet date</t>
         </is>
       </c>
       <c r="B25" s="4">
-        <f>B24/Inputs!$B$22</f>
+        <f>B24-Inputs!$B$19-Inputs!$B$20-Inputs!$B$21-Inputs!$B$22-Inputs!$B$25+Inputs!$B$23+Inputs!$B$24</f>
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>19.15738911847911</v>
+        <v>43635.70864737349</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Value per share (pence)</t>
+          <t>Equity value at valuation date</t>
         </is>
       </c>
       <c r="B26" s="4">
-        <f>B25/Inputs!$B$23*100</f>
+        <f>B25*(1+B17)^Inputs!$B$17-Inputs!$B$18</f>
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1447.588719848807</v>
+        <v>44827.6412113814</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Value per share (USD)</t>
+        </is>
+      </c>
+      <c r="B27" s="4">
+        <f>B26/Inputs!$B$26</f>
+        <v/>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>20.1744559907207</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Value per share (pence)</t>
+        </is>
+      </c>
+      <c r="B28" s="4">
+        <f>B27/Inputs!$B$27*100</f>
+        <v/>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>1524.441286891394</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>Upside vs share price</t>
         </is>
       </c>
-      <c r="B27" s="6">
-        <f>B26/Inputs!$B$24-1</f>
-        <v/>
-      </c>
-      <c r="C27" s="6" t="n">
-        <v>-0.1347347759</v>
+      <c r="B29" s="6">
+        <f>B28/Inputs!$B$28-1</f>
+        <v/>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>-0.0887977962</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phase 3 re-run: Valuation agent with proportionate minorities (1,545p HOLD)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015cJiGSSnTAwJQDY1YEwHLn
</commit_message>
<xml_diff>
--- a/runs/DGE/2026-10-12/valuation/dcf.xlsx
+++ b/runs/DGE/2026-10-12/valuation/dcf.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -745,7 +745,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Minority interests (USD m)</t>
+          <t>Minority interests at book (USD m)</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -760,103 +760,118 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Pension deficit (USD m)</t>
+          <t>Minorities' share of operating profit (proportionate method; blank = use book)</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>0</v>
+        <v>0.02566</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18): net post-employment SURPLUS 627 (XBRL LiabilityAssetOfDefinedBenefitPlans -627); brief rule: 0 if in surplus. Deficit plans alone: 387 (see FLAG)</t>
+          <t>Proportionate minorities (brief: minorities_method). (Profit before exceptional operating items attributable to non-controlling interests 227, Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529) p.210 ROIC table, less EABL's 35% outside shareholders x EABL EBIT 250.2 (Diageo Kenya owns 65% of EABL, 20-F p.164; EBIT as in base_margin) = 139.4) / (operating profit before exceptionals 5,683 - EABL 250.2 = 5,432.8). Simplification: assumes EABL's minorities share EABL's EBIT pro rata.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Associates incl. Moet Hennessy (USD m)</t>
+          <t>Pension deficit (USD m)</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>5284</v>
+        <v>0</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 'Investments in associates': Moet Hennessy 34% at 5,107 (carrying value tested at fair value less costs of disposal, 'sensitive' = little headroom) + others 177</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18): net post-employment SURPLUS 627 (XBRL LiabilityAssetOfDefinedBenefitPlans -627); brief rule: 0 if in surplus. Deficit plans alone: 387 (see FLAG)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Disposal proceeds not in net debt (USD m)</t>
+          <t>Associates incl. Moet Hennessy (USD m)</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>3318.3</v>
+        <v>5284</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>EABL + Kenyan spirits sale to Asahi c.$2.3bn (20-F p.85) + Diageo's 57.21% of USL's RCB sale INR 166.6bn = c.$1.78bn (USL/press, 24 Mar 2026); both gross, before tax and costs, not in net debt at 30 June 2026</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 'Investments in associates': Moet Hennessy 34% at 5,107 (carrying value tested at fair value less costs of disposal, 'sensitive' = little headroom) + others 177</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Restructuring cash still to pay (USD m)</t>
+          <t>Disposal proceeds not in net debt (USD m)</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>850</v>
+        <v>3318.3</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Diageo Capital Markets Day 6-K, 6 Aug 2026 (SEC accession 0001654954-26-007324): c.$800m exceptional cash costs for the operating framework + c.$50m for supply chain in FY27; FY27-29 cumulative free cash flow c.$8bn after c.$850m exceptional cash costs (also 20-F FY26 CEO letter). Pre-tax, undiscounted: any tax relief (up to c.$207m at 24.3%) is not confirmed, so not counted. Not in net debt at 30 June 2026; the forecast is before exceptionals.</t>
+          <t>EABL + Kenyan spirits sale to Asahi c.$2.3bn (20-F p.85) + Diageo's 57.21% of USL's RCB sale INR 166.6bn = c.$1.78bn (USL/press, 24 Mar 2026); both gross, before tax and costs, not in net debt at 30 June 2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ordinary shares (m)</t>
+          <t>Restructuring cash still to pay (USD m)</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>2222</v>
+        <v>850</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) p.188 and XBRL: 2,432m issued - 208m treasury - 2m employee trusts (ordinary shares, NOT ADRs)</t>
+          <t>Diageo Capital Markets Day 6-K, 6 Aug 2026 (SEC accession 0001654954-26-007324): c.$800m exceptional cash costs for the operating framework + c.$50m for supply chain in FY27; FY27-29 cumulative free cash flow c.$8bn after c.$850m exceptional cash costs (also 20-F FY26 CEO letter). Pre-tax, undiscounted: any tax relief (up to c.$207m at 24.3%) is not confirmed, so not counted. Not in net debt at 30 June 2026; the forecast is before exceptionals.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>USD per GBP</t>
+          <t>Ordinary shares (m)</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>1.3234</v>
+        <v>2222</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FRED DEXUSUK (USD per GBP, noon buying rate New York), 2026-10-02</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) p.188 and XBRL: 2,432m issued - 208m treasury - 2m employee trusts (ordinary shares, NOT ADRs)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>USD per GBP</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>1.3234</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>FRED DEXUSUK (USD per GBP, noon buying rate New York), 2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>Share price (pence)</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B29" s="2" t="n">
         <v>1673</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Yahoo Finance DGE.L close (pence, GBp), 2026-10-12</t>
         </is>
@@ -873,7 +888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1438,71 +1453,85 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Equity value at balance sheet date</t>
+          <t>Minority interests deducted</t>
         </is>
       </c>
       <c r="B25" s="4">
-        <f>B24-Inputs!$B$19-Inputs!$B$20-Inputs!$B$21-Inputs!$B$22-Inputs!$B$25+Inputs!$B$23+Inputs!$B$24</f>
+        <f>IF(ISBLANK(Inputs!$B$22),Inputs!$B$21,Inputs!$B$22*B24)</f>
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>43635.70864737349</v>
+        <v>1499.786165891604</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Equity value at valuation date</t>
+          <t>Equity value at balance sheet date</t>
         </is>
       </c>
       <c r="B26" s="4">
-        <f>B25*(1+B17)^Inputs!$B$17-Inputs!$B$18</f>
+        <f>B24-Inputs!$B$19-Inputs!$B$20-B25-Inputs!$B$23-Inputs!$B$26+Inputs!$B$24+Inputs!$B$25</f>
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>44827.6412113814</v>
+        <v>44218.92248148189</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Value per share (USD)</t>
+          <t>Equity value at valuation date</t>
         </is>
       </c>
       <c r="B27" s="4">
-        <f>B26/Inputs!$B$26</f>
+        <f>B26*(1+B17)^Inputs!$B$17-Inputs!$B$18</f>
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>20.1744559907207</v>
+        <v>45426.78584121197</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Value per share (pence)</t>
+          <t>Value per share (USD)</t>
         </is>
       </c>
       <c r="B28" s="4">
-        <f>B27/Inputs!$B$27*100</f>
+        <f>B27/Inputs!$B$27</f>
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1524.441286891394</v>
+        <v>20.44409803834922</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Value per share (pence)</t>
+        </is>
+      </c>
+      <c r="B29" s="4">
+        <f>B28/Inputs!$B$28*100</f>
+        <v/>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>1544.816233818137</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>Upside vs share price</t>
         </is>
       </c>
-      <c r="B29" s="6">
-        <f>B28/Inputs!$B$28-1</f>
-        <v/>
-      </c>
-      <c r="C29" s="6" t="n">
-        <v>-0.0887977962</v>
+      <c r="B30" s="6">
+        <f>B29/Inputs!$B$29-1</f>
+        <v/>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>-0.0766191071</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Phase 4: mid-year discounting (1,627p HOLD), PM bear responses, evidence pack, polished memo
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TQxifsta7TsRzcB6EVYmKB
</commit_message>
<xml_diff>
--- a/runs/DGE/2026-10-12/valuation/dcf.xlsx
+++ b/runs/DGE/2026-10-12/valuation/dcf.xlsx
@@ -1249,23 +1249,23 @@
         </is>
       </c>
       <c r="C13" s="5">
-        <f>1-Inputs!$B$16</f>
+        <f>(0+(1-Inputs!$B$16))/2</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>2-Inputs!$B$16</f>
+        <f>((1-Inputs!$B$16)+(2-Inputs!$B$16))/2</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>3-Inputs!$B$16</f>
+        <f>((2-Inputs!$B$16)+(3-Inputs!$B$16))/2</f>
         <v/>
       </c>
       <c r="F13" s="5">
-        <f>4-Inputs!$B$16</f>
+        <f>((3-Inputs!$B$16)+(4-Inputs!$B$16))/2</f>
         <v/>
       </c>
       <c r="G13" s="5">
-        <f>5-Inputs!$B$16</f>
+        <f>((4-Inputs!$B$16)+(5-Inputs!$B$16))/2</f>
         <v/>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2600.116287717255</v>
+        <v>2707.856642981925</v>
       </c>
     </row>
     <row r="16">
@@ -1391,7 +1391,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>14697.21172715634</v>
+        <v>15306.21633989776</v>
       </c>
     </row>
     <row r="21">
@@ -1429,11 +1429,11 @@
         </is>
       </c>
       <c r="B23" s="4">
-        <f>B22/(1+WACC)^(5-Inputs!$B$16)</f>
+        <f>B22/(1+WACC)^(5-Inputs!$B$16-0.5)</f>
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>43751.19692021715</v>
+        <v>45564.10410506354</v>
       </c>
     </row>
     <row r="24">
@@ -1447,7 +1447,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>58448.40864737349</v>
+        <v>60870.3204449613</v>
       </c>
     </row>
     <row r="25">
@@ -1461,7 +1461,7 @@
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1499.786165891604</v>
+        <v>1561.932422617707</v>
       </c>
     </row>
     <row r="26">
@@ -1475,7 +1475,7 @@
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>44218.92248148189</v>
+        <v>46578.68802234359</v>
       </c>
     </row>
     <row r="27">
@@ -1489,7 +1489,7 @@
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>45426.78584121197</v>
+        <v>47851.0096314929</v>
       </c>
     </row>
     <row r="28">
@@ -1503,7 +1503,7 @@
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>20.44409803834922</v>
+        <v>21.5351078449563</v>
       </c>
     </row>
     <row r="29">
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1544.816233818137</v>
+        <v>1627.256146664372</v>
       </c>
     </row>
     <row r="30">
@@ -1531,7 +1531,7 @@
         <v/>
       </c>
       <c r="C30" s="6" t="n">
-        <v>-0.0766191071</v>
+        <v>-0.0273424108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DGE: re-run valuation after evidence audit (1,808.8p HOLD)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013o7QrhEUYPhCLzn4AyzH1S
</commit_message>
<xml_diff>
--- a/runs/DGE/2026-10-12/valuation/dcf.xlsx
+++ b/runs/DGE/2026-10-12/valuation/dcf.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -460,7 +460,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Base-year net sales ex-EABL (USD m)</t>
+          <t>Base-year net sales, excluding businesses being sold (USD m)</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -580,7 +580,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Risk-free rate (US 10y)</t>
+          <t>Risk-free rate (10-year government bond in USD, the cash-flow currency)</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.05</v>
+        <v>0.042</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -644,11 +644,11 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.29395</v>
+        <v>0.29376</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>net debt 20,482 / (net debt + market cap 49,196 = 2,222m shares x 1673p x 1.3234 USD/GBP)</t>
+          <t>net debt 20,482 / (net debt + market cap 49,240 = 2,224m shares x 1673p x 1.3234 USD/GBP); shares corrected by the evidence audit 15 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Fraction of FY27 elapsed, used in discounting (0 = valued at 30 June)</t>
+          <t>Fraction of the first forecast year elapsed, used in discounting (0 = valued at the balance sheet date)</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -685,7 +685,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Years from 30 June to valuation date (equity roll-forward)</t>
+          <t>Years from the balance sheet date to valuation date (equity roll-forward)</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
@@ -715,22 +715,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Net debt (USD m)</t>
+          <t>Share buybacks after the balance sheet date (USD m)</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>20482</v>
+        <v>0</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 17 p.187: net borrowings 20,482 (INCLUDES lease liabilities 685; EABL/RCB loans of 272 sit in liabilities held for sale)</t>
+          <t>not in this brief's bridge (0)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Lease liabilities not in net debt (USD m)</t>
+          <t>Bridge items already priced at the valuation date, not grown (USD m)</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -738,140 +738,185 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0 because the 685 of lease liabilities is already inside net borrowings (20-F note 17 p.187)</t>
+          <t>not in this brief's bridge (0)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Minority interests at book (USD m)</t>
+          <t>Net debt (USD m)</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>2083</v>
+        <v>20482</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) balance sheet, non-controlling interests at book value (USL 755, other 1,328: p.189)</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 17 p.187: net borrowings 20,482 (INCLUDES lease liabilities 685; EABL/RCB loans of 272 sit in liabilities held for sale)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Minorities' share of operating profit (proportionate method; blank = use book)</t>
+          <t>Lease liabilities not in net debt (USD m)</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>0.02566</v>
+        <v>0</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Proportionate minorities (brief: minorities_method). (Profit before exceptional operating items attributable to non-controlling interests 227, Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529) p.210 ROIC table, less EABL's 35% outside shareholders x EABL EBIT 250.2 (Diageo Kenya owns 65% of EABL, 20-F p.164; EBIT as in base_margin) = 139.4) / (operating profit before exceptionals 5,683 - EABL 250.2 = 5,432.8). Simplification: assumes EABL's minorities share EABL's EBIT pro rata.</t>
+          <t>0 because the 685 of lease liabilities is already inside net borrowings (20-F note 17 p.187)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pension deficit (USD m)</t>
+          <t>Minority interests at book (USD m)</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>0</v>
+        <v>2083</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18): net post-employment SURPLUS 627 (XBRL LiabilityAssetOfDefinedBenefitPlans -627); brief rule: 0 if in surplus. Deficit plans alone: 387 (see FLAG)</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) balance sheet, non-controlling interests at book value (USL 755, other 1,328: p.189)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Associates incl. Moet Hennessy (USD m)</t>
+          <t>Minorities' share of operating profit (proportionate method; blank = use book)</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>5284</v>
+        <v>0.02566</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 'Investments in associates': Moet Hennessy 34% at 5,107 (carrying value tested at fair value less costs of disposal, 'sensitive' = little headroom) + others 177</t>
+          <t>Proportionate minorities (brief: minorities_method). (Profit before exceptional operating items attributable to non-controlling interests 227, Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529) p.210 ROIC table, less EABL's 35% outside shareholders x EABL EBIT 250.2 (Diageo Kenya owns 65% of EABL, 20-F p.164; EBIT as in base_margin) = 139.4) / (operating profit before exceptionals 5,683 - EABL 250.2 = 5,432.8). Simplification: assumes EABL's minorities share EABL's EBIT pro rata.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Disposal proceeds not in net debt (USD m)</t>
+          <t>Pension deficit (USD m)</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>3318.3</v>
+        <v>0</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>EABL + Kenyan spirits sale to Asahi c.$2.3bn (20-F p.85) + Diageo's 57.21% of USL's RCB sale INR 166.6bn = c.$1.78bn (USL/press, 24 Mar 2026); both gross, before tax and costs, not in net debt at 30 June 2026</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18): net post-employment SURPLUS 627 (XBRL LiabilityAssetOfDefinedBenefitPlans -627); brief rule: 0 if in surplus. Deficit plans alone: 387 (see FLAG)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Restructuring cash still to pay (USD m)</t>
+          <t>Associates and equity stakes (USD m)</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>850</v>
+        <v>5284</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Diageo Capital Markets Day 6-K, 6 Aug 2026 (SEC accession 0001654954-26-007324): c.$800m exceptional cash costs for the operating framework + c.$50m for supply chain in FY27; FY27-29 cumulative free cash flow c.$8bn after c.$850m exceptional cash costs (also 20-F FY26 CEO letter). Pre-tax, undiscounted: any tax relief (up to c.$207m at 24.3%) is not confirmed, so not counted. Not in net debt at 30 June 2026; the forecast is before exceptionals.</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) note 'Investments in associates': Moet Hennessy 34% at 5,107 (carrying value tested at fair value less costs of disposal, 'sensitive' = little headroom) + others 177</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ordinary shares (m)</t>
+          <t>Disposal proceeds not in net debt (USD m)</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>2222</v>
+        <v>3318.3</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) p.188 and XBRL: 2,432m issued - 208m treasury - 2m employee trusts (ordinary shares, NOT ADRs)</t>
+          <t>EABL + Kenyan spirits sale to Asahi c.$2.3bn (20-F p.85) + Diageo's 57.21% of USL's RCB sale INR 166.6bn = c.$1.78bn (USL/press, 24 Mar 2026); both gross, before tax and costs, not in net debt at 30 June 2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>USD per GBP</t>
+          <t>Restructuring cash still to pay (USD m)</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>1.3234</v>
+        <v>850</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FRED DEXUSUK (USD per GBP, noon buying rate New York), 2026-10-02</t>
+          <t>Diageo Capital Markets Day 6-K, 6 Aug 2026 (SEC accession 0001654954-26-007324): c.$800m exceptional cash costs for the operating framework + c.$50m for supply chain in FY27; FY27-29 cumulative free cash flow c.$8bn after c.$850m exceptional cash costs (also 20-F FY26 CEO letter). Pre-tax, undiscounted: any tax relief (up to c.$207m at 24.3%) is not confirmed, so not counted. Not in net debt at 30 June 2026; the forecast is before exceptionals.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Contingent liabilities assumed paid, e.g. a lost tax case (USD m)</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>not in this brief's bridge (0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Ordinary shares (m)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>2224</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) p.188 and XBRL: 2,432m issued - 208m own shares (treasury AND employee trusts, note 18(c)) = 2,224m ordinary shares (NOT ADRs); cross-check: weighted average shares excluding own shares 2,224m. Evidence audit 15 Oct 2026 (was 2,222m: trusts deducted twice). Basic count; dilutive options (+7m) not added, the desk's convention</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>USD per GBP</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>1.3234</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>FRED DEXUSUK (USD per GBP, noon buying rate New York), 2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Share price (pence)</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B32" s="2" t="n">
         <v>1673</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Yahoo Finance DGE.L close (pence, GBp), 2026-10-12</t>
         </is>
@@ -1323,7 +1368,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2707.856642981925</v>
+        <v>2769.531499082056</v>
       </c>
     </row>
     <row r="16">
@@ -1349,7 +1394,7 @@
         <v/>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.100205</v>
+        <v>0.0925242</v>
       </c>
     </row>
     <row r="18">
@@ -1377,7 +1422,7 @@
         <v/>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.08459049358000001</v>
+        <v>0.07917609811200001</v>
       </c>
     </row>
     <row r="20">
@@ -1391,7 +1436,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>15306.21633989776</v>
+        <v>15490.0355213282</v>
       </c>
     </row>
     <row r="21">
@@ -1419,7 +1464,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>65662.7256636308</v>
+        <v>71670.6237101834</v>
       </c>
     </row>
     <row r="23">
@@ -1433,7 +1478,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>45564.10410506354</v>
+        <v>50865.78524866833</v>
       </c>
     </row>
     <row r="24">
@@ -1447,7 +1492,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>60870.3204449613</v>
+        <v>66355.82076999653</v>
       </c>
     </row>
     <row r="25">
@@ -1457,11 +1502,11 @@
         </is>
       </c>
       <c r="B25" s="4">
-        <f>IF(ISBLANK(Inputs!$B$22),Inputs!$B$21,Inputs!$B$22*B24)</f>
+        <f>IF(ISBLANK(Inputs!$B$24),Inputs!$B$23,Inputs!$B$24*B24)</f>
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1561.932422617707</v>
+        <v>1702.690360958111</v>
       </c>
     </row>
     <row r="26">
@@ -1471,11 +1516,11 @@
         </is>
       </c>
       <c r="B26" s="4">
-        <f>B24-Inputs!$B$19-Inputs!$B$20-B25-Inputs!$B$23-Inputs!$B$26+Inputs!$B$24+Inputs!$B$25</f>
+        <f>B24-Inputs!$B$21-Inputs!$B$22-B25-Inputs!$B$25-Inputs!$B$28-Inputs!$B$29+Inputs!$B$26+Inputs!$B$27</f>
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>46578.68802234359</v>
+        <v>51923.43040903842</v>
       </c>
     </row>
     <row r="27">
@@ -1485,11 +1530,11 @@
         </is>
       </c>
       <c r="B27" s="4">
-        <f>B26*(1+B17)^Inputs!$B$17-Inputs!$B$18</f>
+        <f>(B26-Inputs!$B$20)*(1+B17)^Inputs!$B$17+Inputs!$B$20-Inputs!$B$18-Inputs!$B$19</f>
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>47851.0096314929</v>
+        <v>53236.39317352109</v>
       </c>
     </row>
     <row r="28">
@@ -1499,11 +1544,11 @@
         </is>
       </c>
       <c r="B28" s="4">
-        <f>B27/Inputs!$B$27</f>
+        <f>B27/Inputs!$B$30</f>
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>21.5351078449563</v>
+        <v>23.93722714636739</v>
       </c>
     </row>
     <row r="29">
@@ -1513,11 +1558,11 @@
         </is>
       </c>
       <c r="B29" s="4">
-        <f>B28/Inputs!$B$28*100</f>
+        <f>B28/Inputs!$B$31*100</f>
         <v/>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1627.256146664372</v>
+        <v>1808.767352755584</v>
       </c>
     </row>
     <row r="30">
@@ -1527,11 +1572,11 @@
         </is>
       </c>
       <c r="B30" s="6">
-        <f>B29/Inputs!$B$29-1</f>
+        <f>B29/Inputs!$B$32-1</f>
         <v/>
       </c>
       <c r="C30" s="6" t="n">
-        <v>-0.0273424108</v>
+        <v>0.0811520339</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalising runs after PM bear responses (in progress)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013o7QrhEUYPhCLzn4AyzH1S
</commit_message>
<xml_diff>
--- a/runs/DGE/2026-10-12/valuation/dcf.xlsx
+++ b/runs/DGE/2026-10-12/valuation/dcf.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.06211688111691262</v>
+        <v>0.062167019144524</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -644,11 +644,11 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.29376</v>
+        <v>0.29311</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>net debt 20,482 / (net debt + market cap 49,240 = 2,224m shares x 1673p x 1.3234 USD/GBP); shares corrected by the evidence audit 15 Oct 2026</t>
+          <t>net debt 20,482 / (net debt + market cap 49,395 = 2,231m diluted shares x 1673p x 1.3234 USD/GBP); PM decision 15 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -884,11 +884,11 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>2224</v>
+        <v>2231</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18) p.188 and XBRL: 2,432m issued - 208m own shares (treasury AND employee trusts, note 18(c)) = 2,224m ordinary shares (NOT ADRs); cross-check: weighted average shares excluding own shares 2,224m. Evidence audit 15 Oct 2026 (was 2,222m: trusts deducted twice). Basic count; dilutive options (+7m) not added, the desk's convention</t>
+          <t>Diageo Form 20-F FY26 (SEC accession 0001628280-26-057529, filed 2026-08-18): 2,432m issued - 208m own shares (treasury AND employee trusts, note 18(c)) = 2,224m basic + 7m dilutive potential ordinary shares (EPS note, diluted weighted average) = 2,231m ordinary shares (NOT ADRs). PM decision 15 Oct 2026 (evidence audit bear responses, D3)</t>
         </is>
       </c>
     </row>
@@ -998,10 +998,10 @@
         <v>0.025</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="3">
@@ -1035,7 +1035,7 @@
         <v/>
       </c>
       <c r="I3" s="4" t="n">
-        <v>20425.14652985625</v>
+        <v>20030.46700882499</v>
       </c>
     </row>
     <row r="4">
@@ -1092,7 +1092,7 @@
         <v/>
       </c>
       <c r="I5" s="4" t="n">
-        <v>6456.414518235197</v>
+        <v>6340.544504450842</v>
       </c>
     </row>
     <row r="6">
@@ -1257,7 +1257,7 @@
         <v/>
       </c>
       <c r="I11" s="4" t="n">
-        <v>3902.30975406807</v>
+        <v>3905.274736223222</v>
       </c>
     </row>
     <row r="12">
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2769.531499082056</v>
+        <v>2771.294472542121</v>
       </c>
     </row>
     <row r="16">
@@ -1422,7 +1422,7 @@
         <v/>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.07917609811200001</v>
+        <v>0.07920563333200001</v>
       </c>
     </row>
     <row r="20">
@@ -1436,7 +1436,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>15490.0355213282</v>
+        <v>15519.25996953602</v>
       </c>
     </row>
     <row r="21">
@@ -1450,7 +1450,7 @@
         <v/>
       </c>
       <c r="C21" s="4" t="n">
-        <v>4241.187860422046</v>
+        <v>4165.073401776124</v>
       </c>
     </row>
     <row r="22">
@@ -1464,7 +1464,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>71670.6237101834</v>
+        <v>70349.27535392054</v>
       </c>
     </row>
     <row r="23">
@@ -1478,7 +1478,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>50865.78524866833</v>
+        <v>49921.85469752825</v>
       </c>
     </row>
     <row r="24">
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>66355.82076999653</v>
+        <v>65441.11466706427</v>
       </c>
     </row>
     <row r="25">
@@ -1506,7 +1506,7 @@
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1702.690360958111</v>
+        <v>1679.219002356869</v>
       </c>
     </row>
     <row r="26">
@@ -1520,7 +1520,7 @@
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>51923.43040903842</v>
+        <v>51032.1956647074</v>
       </c>
     </row>
     <row r="27">
@@ -1534,7 +1534,7 @@
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>53236.39317352109</v>
+        <v>52322.62220566821</v>
       </c>
     </row>
     <row r="28">
@@ -1548,7 +1548,7 @@
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>23.93722714636739</v>
+        <v>23.45254244987369</v>
       </c>
     </row>
     <row r="29">
@@ -1562,7 +1562,7 @@
         <v/>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1808.767352755584</v>
+        <v>1772.143150209589</v>
       </c>
     </row>
     <row r="30">
@@ -1576,7 +1576,7 @@
         <v/>
       </c>
       <c r="C30" s="6" t="n">
-        <v>0.0811520339</v>
+        <v>0.0592606995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DGE: exact Damodaran industry beta 0.7250, not a rounded 0.73 (HOLD 1,780.2p)
Source check of 15 Oct 2026 against the PM's uploaded betaGlobal.xls: Beverage
(Alcoholic) unlevered beta corrected for cash is 0.7250. Relevered at Diageo's
current D/E: beta 0.9526 (was 0.9601). Valuation, bridge, sanity, steps and bear
re-run; memo and PDF updated. Fair value 1,772.1p -> 1,780.2p GBp, still HOLD.
Adds the source-check report (docs/audit-2026-10-15/source-check-2026-10-15.md).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AFuQYzLJi8aQ8rMuggN6sm
</commit_message>
<xml_diff>
--- a/runs/DGE/2026-10-12/valuation/dcf.xlsx
+++ b/runs/DGE/2026-10-12/valuation/dcf.xlsx
@@ -614,11 +614,11 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.9601</v>
+        <v>0.9526</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Risk agent, bottom-up: Damodaran global alcoholic beverages unlevered beta 0.73 (Jan 2026, cash-corrected) relevered at Diageo D/E 0.416, tax 24.3%. See risk/beta_evidence.json</t>
+          <t>Risk agent, bottom-up: Damodaran global alcoholic beverages unlevered beta corrected for cash 0.7250 (betaGlobal.xls, 5 Jan 2026, 217 firms) relevered at Diageo market D/E 0.4146 (debt weight 0.29311), tax 24.3%. Source check 15 Oct 2026: was 0.9601 from a rounded 0.73 (mistakes log row 33). See risk/beta_evidence.json</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2771.294472542121</v>
+        <v>2773.869013689381</v>
       </c>
     </row>
     <row r="16">
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.0925242</v>
+        <v>0.09220920000000001</v>
       </c>
     </row>
     <row r="18">
@@ -1422,7 +1422,7 @@
         <v/>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0.07920563333200001</v>
+        <v>0.07898296298200001</v>
       </c>
     </row>
     <row r="20">
@@ -1436,7 +1436,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>15519.25996953602</v>
+        <v>15526.92454144778</v>
       </c>
     </row>
     <row r="21">
@@ -1464,7 +1464,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>70349.27535392054</v>
+        <v>70614.8553955689</v>
       </c>
     </row>
     <row r="23">
@@ -1478,7 +1478,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>49921.85469752825</v>
+        <v>50156.87051952619</v>
       </c>
     </row>
     <row r="24">
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>65441.11466706427</v>
+        <v>65683.79506097398</v>
       </c>
     </row>
     <row r="25">
@@ -1506,7 +1506,7 @@
         <v/>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1679.219002356869</v>
+        <v>1685.446181264592</v>
       </c>
     </row>
     <row r="26">
@@ -1520,7 +1520,7 @@
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>51032.1956647074</v>
+        <v>51268.64887970939</v>
       </c>
     </row>
     <row r="27">
@@ -1534,7 +1534,7 @@
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>52322.62220566821</v>
+        <v>52560.77711201133</v>
       </c>
     </row>
     <row r="28">
@@ -1548,7 +1548,7 @@
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>23.45254244987369</v>
+        <v>23.55929050291857</v>
       </c>
     </row>
     <row r="29">
@@ -1562,7 +1562,7 @@
         <v/>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1772.143150209589</v>
+        <v>1780.209347356701</v>
       </c>
     </row>
     <row r="30">
@@ -1576,7 +1576,7 @@
         <v/>
       </c>
       <c r="C30" s="6" t="n">
-        <v>0.0592606995</v>
+        <v>0.0640820964</v>
       </c>
     </row>
   </sheetData>

</xml_diff>